<commit_message>
Update pipeline data and documentation for May 2026 refresh
- Refresh lung-centers.txt and lung-transplants.csv with May 7 2026 scrape (55 centers, 2005-2026)
- Update CLAUDE.md: clarify routine (Step 3 only) vs. full pipeline refresh with timing notes
- Add claudeprompt1.1.txt: session context supplement for next conversation
- Update .gitignore: exclude .DS_Store and settings.local.json

Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Reports/lung-transplants.xlsx
+++ b/Reports/lung-transplants.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tsk/Desktop/Automation Projects/Playwright_projects/Reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D416AC-2E9D-4741-89F7-1AF466875224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D4832B-81AA-7545-9DAA-129B430C0268}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LungstodateMar2026" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>